<commit_message>
Populate Finland admissions data and source tracking
</commit_message>
<xml_diff>
--- a/excel/universities/aalto-university.xlsx
+++ b/excel/universities/aalto-university.xlsx
@@ -115,7 +115,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.aalto.fi/en/study-options</t>
+          <t xml:space="preserve">https://www.aalto.fi/en/admission-services/masters-admissions</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -125,27 +125,27 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t xml:space="preserve">University-wide international master's admissions</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Autumn</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Autumn</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Programme-specific</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fill program-specific information here</t>
+          <t xml:space="preserve">Main annual master's intake runs in December-January; applicants may apply to up to two study options.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -229,37 +229,37 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t xml:space="preserve">University-wide international master's admissions</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Autumn</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-01</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-02</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Autumn</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.aalto.fi/en/study-options</t>
+          <t xml:space="preserve">https://www.aalto.fi/en/admission-services/masters-admissions</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verify annual deadlines</t>
+          <t xml:space="preserve">Document upload deadline 2026-01-09; results published 2026-04-08.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -275,7 +275,7 @@
 
 <file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -333,30 +333,156 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">University-wide international master's admissions</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Passport</t>
+          <t xml:space="preserve">Degree certificate</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t xml:space="preserve">If graduated</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Upload with official translations when required.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/admission-services/masters-admissions</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Master</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">University-wide international master's admissions</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transcript of records</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.aalto.fi/en/study-options</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Upload by 2026-01-09 if applying for autumn 2026 intake.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/admission-services/masters-admissions</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Master</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">University-wide international master's admissions</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proof of language proficiency</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accepted methods are listed on Aalto language requirements page.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/admission-services/language-requirements-in-masters-admissions</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Master</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">University-wide international master's admissions</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Study-option-specific documents</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check programme</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Programme page may require GRE or GMAT or portfolio depending on field.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/admission-services/masters-admissions</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-03-14</t>
         </is>
@@ -369,7 +495,7 @@
 
 <file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -420,15 +546,30 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t xml:space="preserve">citation_source</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">citation_last_checked</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t xml:space="preserve">official_profile_url</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t xml:space="preserve">email</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">notes</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
         <is>
           <t xml:space="preserve">last_verified</t>
         </is>
@@ -442,12 +583,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Department Name</t>
+          <t xml:space="preserve">Department of Information and Communications Engineering</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Professor Name</t>
+          <t xml:space="preserve">Antti Oulasvirta</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -457,7 +598,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research Area 1; Research Area 2</t>
+          <t xml:space="preserve">Human-computer interaction; User interfaces; Human factors; Interactive AI; Computational modeling</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -472,25 +613,40 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">14763</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">63</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.aalto.fi/</t>
+          <t xml:space="preserve">Research.com profile summary</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2026-03-14</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/people/antti-oulasvirta</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">antti.oulasvirta@aalto.fi</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto official profile does not expose ResearchGate or Google Scholar links directly on the page snapshot used here.</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-03-14</t>
         </is>

</xml_diff>

<commit_message>
Add department datasets and align professor mapping
</commit_message>
<xml_diff>
--- a/excel/universities/aalto-university.xlsx
+++ b/excel/universities/aalto-university.xlsx
@@ -20,7 +20,8 @@
     <sheet name="UniversityInfo" sheetId="1" r:id="rId1"/>
     <sheet name="Deadlines" sheetId="2" r:id="rId2"/>
     <sheet name="Documents" sheetId="3" r:id="rId3"/>
-    <sheet name="Professors" sheetId="4" r:id="rId4"/>
+    <sheet name="Departments" sheetId="4" r:id="rId4"/>
+    <sheet name="Professors" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -495,7 +496,7 @@
 
 <file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,70 +507,40 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t xml:space="preserve">department_name</t>
+          <t xml:space="preserve">unit_type</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t xml:space="preserve">professor_name</t>
+          <t xml:space="preserve">unit_name</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t xml:space="preserve">title</t>
+          <t xml:space="preserve">parent_unit</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t xml:space="preserve">research_areas</t>
+          <t xml:space="preserve">campus_or_city</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t xml:space="preserve">researchgate_url</t>
+          <t xml:space="preserve">focus_areas</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t xml:space="preserve">google_scholar_url</t>
+          <t xml:space="preserve">official_url</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t xml:space="preserve">citation_count</t>
+          <t xml:space="preserve">notes</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">h_index</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">citation_source</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">citation_last_checked</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">official_profile_url</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">email</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">notes</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
         <is>
           <t xml:space="preserve">last_verified</t>
         </is>
@@ -583,6 +554,1362 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t xml:space="preserve">School</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Arts, Design and Architecture</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Art; Design; Architecture; Media</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/school-of-arts-design-and-architecture</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto school page.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Architecture</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Arts, Design and Architecture</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Architecture</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-architecture</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Art and Media</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Arts, Design and Architecture</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Art; Media; Visual culture</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-art-and-media</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Design</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Arts, Design and Architecture</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Design</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-design</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Film</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Arts, Design and Architecture</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Film; Television; Scenography</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-film</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Business</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Business; Economics; Management</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/school-of-business</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto school page.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Accounting and Business Law</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Business</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accounting; Business law</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-accounting-and-business-law</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Economics</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Business</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Economics</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-economics</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Finance</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Business</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Finance</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-finance</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Information and Service Management</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Business</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Information systems; Service management</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-information-and-service-management</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Management Studies</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Business</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Management; Organization</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-management-studies</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Marketing</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Business</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marketing</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-marketing</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Chemical Engineering</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chemical engineering; Materials; Bioproducts</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/school-of-chemical-engineering</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto school page.</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Bioproducts and Biosystems</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Chemical Engineering</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bioproducts; Biosystems</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-bioproducts-and-biosystems</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Chemistry and Materials Science</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Chemical Engineering</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chemistry; Materials science</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-chemistry-and-materials-science</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Chemical and Metallurgical Engineering</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Chemical Engineering</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chemical engineering; Metallurgy</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-chemical-and-metallurgical-engineering</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrical engineering; Electronics; Automation</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/school-of-electrical-engineering</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto school page.</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Engineering</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Engineering; Built environment; Energy</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/school-of-engineering</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto school page.</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Built Environment</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Engineering</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Built environment; Real estate; Water</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-built-environment</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Civil Engineering</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Engineering</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Civil engineering</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-civil-engineering</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Energy and Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Engineering</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Energy; Mechanical engineering</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-energy-and-mechanical-engineering</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Science</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Computer science; Mathematics; Physics; Industrial engineering</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/school-of-science</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto school page.</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Applied Physics</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Science</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Applied physics</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-applied-physics</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Computer Science</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Science</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Computer science</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-computer-science</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Industrial Engineering and Management</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Science</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Industrial engineering; Management</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-industrial-engineering-and-management</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Mathematics and Systems Analysis</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Science</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mathematics; Systems analysis</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-mathematics-and-systems-analysis</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Neuroscience and Biomedical Engineering</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Science</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espoo</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Neuroscience; Biomedical engineering</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/department-of-neuroscience-and-biomedical-engineering</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto department page.</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">university_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">department_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">professor_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">research_areas</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">researchgate_url</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">google_scholar_url</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">citation_count</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">h_index</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">citation_source</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">citation_last_checked</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">official_profile_url</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">email</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">notes</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">last_verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Department of Information and Communications Engineering</t>
         </is>
       </c>
@@ -649,6 +1976,160 @@
       <c r="O2" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Computer Science</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Samuel Kaski</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Professor</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Artificial intelligence; Machine learning; Probabilistic modeling; Computational health</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto official profile</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/people/samuel-kaski</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto profile used for department and research-focus mapping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto University</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Computer Science</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aristides Gionis</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Professor</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data mining; Algorithms; Network analysis; Machine learning</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aalto official profile</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.aalto.fi/en/people/aristides-gionis</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Aalto profile used for department and research-focus mapping.</t>
         </is>
       </c>
     </row>

</xml_diff>